<commit_message>
add 2 glava and modificate images
</commit_message>
<xml_diff>
--- a/Documens/task_spreading.xlsx
+++ b/Documens/task_spreading.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1\Documents\GitHub\webApplication_development_2026\Documens\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C55A79A-295C-4DA0-8D86-C8F9A88ED3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45DFC560-203D-4F09-8DB2-792CA2969100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -340,7 +340,7 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -363,6 +363,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFCC99FF"/>
         <bgColor rgb="FFCC99FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -393,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -432,15 +444,33 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -754,13 +784,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -786,7 +816,7 @@
       <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="18" t="s">
         <v>49</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -798,10 +828,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="18" t="s">
         <v>50</v>
       </c>
       <c r="D4" s="11"/>
@@ -811,10 +841,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="18" t="s">
         <v>51</v>
       </c>
       <c r="D5" s="11"/>
@@ -824,10 +854,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="18" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -839,10 +869,10 @@
     </row>
     <row r="7" spans="1:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="19" t="s">
         <v>55</v>
       </c>
       <c r="D7" s="4"/>
@@ -852,10 +882,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="20" t="s">
         <v>56</v>
       </c>
       <c r="D8" s="4"/>
@@ -865,10 +895,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -880,10 +910,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="19" t="s">
         <v>58</v>
       </c>
       <c r="D10" s="3"/>
@@ -893,10 +923,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="20" t="s">
         <v>59</v>
       </c>
       <c r="D11" s="3"/>
@@ -908,10 +938,10 @@
       <c r="A12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="18" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -923,10 +953,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="22" t="s">
         <v>61</v>
       </c>
       <c r="D13" s="3"/>
@@ -936,10 +966,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="20" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="3"/>
@@ -949,10 +979,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="18" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="4" t="s">
@@ -964,10 +994,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="23" t="s">
         <v>63</v>
       </c>
       <c r="D16" s="4"/>
@@ -977,10 +1007,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="18" t="s">
         <v>71</v>
       </c>
       <c r="D17" s="4"/>
@@ -990,10 +1020,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="18" t="s">
         <v>68</v>
       </c>
       <c r="D18" s="4" t="s">
@@ -1005,10 +1035,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="18" t="s">
         <v>73</v>
       </c>
       <c r="D19" s="3"/>
@@ -1018,10 +1048,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="23" t="s">
         <v>72</v>
       </c>
       <c r="D20" s="3"/>
@@ -1031,10 +1061,10 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D21" s="4" t="s">
@@ -1046,10 +1076,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="22" t="s">
         <v>74</v>
       </c>
       <c r="D22" s="3"/>
@@ -1059,10 +1089,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="20" t="s">
         <v>75</v>
       </c>
       <c r="D23" s="3"/>
@@ -1131,7 +1161,7 @@
       <c r="B28" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="15" t="s">
         <v>80</v>
       </c>
       <c r="D28" s="3"/>
@@ -1144,7 +1174,7 @@
       <c r="B29" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="15" t="s">
         <v>81</v>
       </c>
       <c r="D29" s="3"/>

</xml_diff>